<commit_message>
Add report date to the bottom
</commit_message>
<xml_diff>
--- a/api/templates/module_status_report/en.xlsx
+++ b/api/templates/module_status_report/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\opewix\dev\sysone\sources\aspect\api\templates\module_status_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16920F80-F663-44CD-B35B-B2E24702380D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC9694D7-C15A-4E4C-BD79-C0831A3D3F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Module Status Report</t>
   </si>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t>&lt;activeModuleBays&gt;</t>
+  </si>
+  <si>
+    <t>* Modules marked Do Not Use on &lt;ReportDate&gt;</t>
   </si>
 </sst>
 </file>
@@ -205,7 +208,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -221,7 +224,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -604,7 +606,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" customWidth="1"/>
@@ -701,8 +703,13 @@
       <c r="H8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="9" t="s">
+      <c r="I8" s="6" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>